<commit_message>
Update scalper, price watcher, Excel builder, and trade journal
- scalper-run.js: fix 24/7 crypto market hours, auth header guard for demo mode, iterative safety-check-log saves
- scripts/price_watcher.js: new persistent watcher using single watchlist DOM call
- scripts/update_excel.js: add forex account to Portfolio sheet, combined balance view
- src/connection.js: keepalive ping, exponential backoff reconnect
- trade-journal.json: add forex_account block
- .gitignore: exclude .claude/, .obsidian/, Excel lock files

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/trades/trade-journal.xlsx
+++ b/trades/trade-journal.xlsx
@@ -15,7 +15,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="43">
   <si>
-    <t>🤖 Claude Trade Journal  |  Started: 2026-04-09  |  Target: 2x by 2026-04-19  |  Last Updated: 9/4/2026, 4:44:46 pm IST</t>
+    <t>🤖 Claude Trade Journal  |  Started: 2026-04-09  |  Target: 2x by 2026-04-25  |  Last Updated: 10/4/2026, 4:16:24 pm IST</t>
   </si>
   <si>
     <t>#</t>
@@ -96,7 +96,7 @@
     <t>🏁  Target Date</t>
   </si>
   <si>
-    <t>2026-04-19</t>
+    <t>2026-04-25</t>
   </si>
   <si>
     <t>⏳  Days Remaining</t>
@@ -132,7 +132,7 @@
     <t>🕐  Last Updated</t>
   </si>
   <si>
-    <t>9/4/2026, 4:44:46 pm IST</t>
+    <t>10/4/2026, 4:16:24 pm IST</t>
   </si>
   <si>
     <t>Note</t>
@@ -151,7 +151,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="₹#,##0.00"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -170,10 +170,6 @@
     <font>
       <b/>
       <color rgb="FF00B050"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFF0000"/>
     </font>
     <font>
       <b/>
@@ -257,7 +253,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -280,16 +276,13 @@
     <xf numFmtId="10" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -298,19 +291,19 @@
     <xf numFmtId="10" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -319,16 +312,16 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -834,7 +827,7 @@
         <v>66.8</v>
       </c>
       <c r="G4" s="6">
-        <v>65.4</v>
+        <v>66.8</v>
       </c>
       <c r="H4" s="6">
         <v>78</v>
@@ -849,77 +842,77 @@
         <v>4676</v>
       </c>
       <c r="L4" s="6">
-        <v>-97.9999999999994</v>
-      </c>
-      <c r="M4" s="8">
-        <v>-0.020958083832335203</v>
+        <v>0</v>
+      </c>
+      <c r="M4" s="7">
+        <v>0</v>
       </c>
       <c r="N4" s="3">
         <v>1.93</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="9">
+      <c r="A5" s="8">
         <v>1</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="12">
+      <c r="F5" s="11">
         <v>334.09</v>
       </c>
-      <c r="G5" s="12">
+      <c r="G5" s="11">
         <v>334.5</v>
       </c>
-      <c r="H5" s="12">
+      <c r="H5" s="11">
         <v>370</v>
       </c>
-      <c r="I5" s="12">
+      <c r="I5" s="11">
         <v>310</v>
       </c>
-      <c r="J5" s="9">
+      <c r="J5" s="8">
         <v>29</v>
       </c>
-      <c r="K5" s="12">
+      <c r="K5" s="11">
         <v>9688.61</v>
       </c>
-      <c r="L5" s="12">
+      <c r="L5" s="11">
         <v>11.890000000000725</v>
       </c>
-      <c r="M5" s="13">
+      <c r="M5" s="12">
         <v>0.0012272142237122483</v>
       </c>
-      <c r="N5" s="9">
+      <c r="N5" s="8">
         <v>1.49</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="14"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="14"/>
-      <c r="J6" s="14"/>
-      <c r="L6" s="15">
-        <v>-86.10999999999868</v>
-      </c>
-      <c r="M6" s="16">
-        <v>-0.008610999999999867</v>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13"/>
+      <c r="I6" s="13"/>
+      <c r="J6" s="13"/>
+      <c r="L6" s="14">
+        <v>11.890000000000725</v>
+      </c>
+      <c r="M6" s="15">
+        <v>0.0011890000000000726</v>
       </c>
     </row>
   </sheetData>
@@ -947,10 +940,10 @@
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="17" t="s">
         <v>23</v>
       </c>
     </row>
@@ -960,27 +953,27 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="19" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="19" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="20">
-        <v>10</v>
+      <c r="B6" s="19">
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
@@ -989,43 +982,43 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="B8" s="22">
+      <c r="B8" s="21">
         <v>10000</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="22">
-        <v>20000</v>
+      <c r="B9" s="21">
+        <v>40000</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="23">
-        <v>9913.890000000001</v>
+      <c r="B10" s="22">
+        <v>10011.890000000001</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="23">
-        <v>-86.10999999999868</v>
+      <c r="B11" s="22">
+        <v>11.890000000000725</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="24">
-        <v>-0.008610999999999876</v>
+      <c r="B12" s="23">
+        <v>0.0011890000000001238</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
@@ -1034,34 +1027,34 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="B14" s="20">
+      <c r="B14" s="19">
         <v>3</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="B15" s="20">
+      <c r="B15" s="19">
         <v>2</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B16" s="25">
+      <c r="B16" s="24">
         <v>1</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="26" t="s">
+      <c r="A17" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="B17" s="27">
+      <c r="B17" s="26">
         <v>0</v>
       </c>
     </row>
@@ -1071,10 +1064,10 @@
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="B19" s="20" t="s">
+      <c r="B19" s="19" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1102,18 +1095,18 @@
       </c>
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="28" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="30" t="s">
+      <c r="A3" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="31" t="s">
+      <c r="B3" s="30" t="s">
         <v>42</v>
       </c>
     </row>

</xml_diff>